<commit_message>
SPM-84: Event Coordinator Lead – rename role and view assignments
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-21_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-21_Test_Cases.xlsx
@@ -34,7 +34,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -63,6 +63,9 @@
       <name val="Arial"/>
       <color theme="1"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
     </font>
   </fonts>
   <fills count="4">
@@ -148,7 +151,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -198,6 +201,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -490,12 +496,12 @@
   </cols>
   <sheetData>
     <row r="1" ht="30.75" customHeight="1" s="20">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="23" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="23" t="inlineStr">
         <is>
           <t>SPM-21: As a ConnectSphere user, I want to securely log in to the system so that I can access functionality appropriate to my role</t>
         </is>
@@ -507,32 +513,32 @@
     </row>
     <row r="2"/>
     <row r="3">
-      <c r="A3" s="1" t="inlineStr">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B3" s="1" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="C3" s="1" t="inlineStr">
+      <c r="C3" s="23" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D3" s="1" t="inlineStr">
+      <c r="D3" s="23" t="inlineStr">
         <is>
           <t>Linked AC</t>
         </is>
       </c>
-      <c r="E3" s="1" t="inlineStr">
+      <c r="E3" s="23" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F3" s="1" t="inlineStr">
+      <c r="F3" s="23" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
@@ -559,27 +565,27 @@
           <t>TC01</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC01</t>
         </is>
       </c>
-      <c r="C4" s="16" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>Valid credentials sign the user in and open the dashboard</t>
         </is>
       </c>
-      <c r="D4" s="16" t="inlineStr">
+      <c r="D4" s="24" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E4" s="16" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F4" s="16" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
@@ -598,27 +604,27 @@
           <t>TC02</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC02</t>
         </is>
       </c>
-      <c r="C5" s="16" t="inlineStr">
+      <c r="C5" s="24" t="inlineStr">
         <is>
           <t>The signed-in chrome appears immediately, without a manual refresh</t>
         </is>
       </c>
-      <c r="D5" s="16" t="inlineStr">
+      <c r="D5" s="24" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E5" s="16" t="inlineStr">
+      <c r="E5" s="24" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -637,27 +643,27 @@
           <t>TC03</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC03</t>
         </is>
       </c>
-      <c r="C6" s="16" t="inlineStr">
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>After signing in, the user is returned to the page they first asked for</t>
         </is>
       </c>
-      <c r="D6" s="16" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E6" s="16" t="inlineStr">
+      <c r="E6" s="24" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -676,27 +682,27 @@
           <t>TC04</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC04</t>
         </is>
       </c>
-      <c r="C7" s="16" t="inlineStr">
+      <c r="C7" s="24" t="inlineStr">
         <is>
           <t>The session survives a browser refresh</t>
         </is>
       </c>
-      <c r="D7" s="16" t="inlineStr">
+      <c r="D7" s="24" t="inlineStr">
         <is>
           <t>AC1, AC3</t>
         </is>
       </c>
-      <c r="E7" s="16" t="inlineStr">
+      <c r="E7" s="24" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="F7" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -715,27 +721,27 @@
           <t>TC05</t>
         </is>
       </c>
-      <c r="B8" s="16" t="inlineStr">
+      <c r="B8" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC05</t>
         </is>
       </c>
-      <c r="C8" s="16" t="inlineStr">
+      <c r="C8" s="24" t="inlineStr">
         <is>
           <t>A wrong password is refused with an error message</t>
         </is>
       </c>
-      <c r="D8" s="16" t="inlineStr">
+      <c r="D8" s="24" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="E8" s="16" t="inlineStr">
+      <c r="E8" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="24" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
@@ -754,27 +760,27 @@
           <t>TC06</t>
         </is>
       </c>
-      <c r="B9" s="16" t="inlineStr">
+      <c r="B9" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC06</t>
         </is>
       </c>
-      <c r="C9" s="16" t="inlineStr">
+      <c r="C9" s="24" t="inlineStr">
         <is>
           <t>An unknown email is refused with the same message as a wrong password</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D9" s="24" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="E9" s="16" t="inlineStr">
+      <c r="E9" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="F9" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -793,27 +799,27 @@
           <t>TC07</t>
         </is>
       </c>
-      <c r="B10" s="16" t="inlineStr">
+      <c r="B10" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC07</t>
         </is>
       </c>
-      <c r="C10" s="16" t="inlineStr">
+      <c r="C10" s="24" t="inlineStr">
         <is>
           <t>An email that is not a valid address is refused with a message naming the problem</t>
         </is>
       </c>
-      <c r="D10" s="16" t="inlineStr">
+      <c r="D10" s="24" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="E10" s="16" t="inlineStr">
+      <c r="E10" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="24" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
@@ -832,27 +838,27 @@
           <t>TC08</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC08</t>
         </is>
       </c>
-      <c r="C11" s="16" t="inlineStr">
+      <c r="C11" s="24" t="inlineStr">
         <is>
           <t>An empty password is refused with a message naming the problem</t>
         </is>
       </c>
-      <c r="D11" s="16" t="inlineStr">
+      <c r="D11" s="24" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="E11" s="16" t="inlineStr">
+      <c r="E11" s="24" t="inlineStr">
         <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F11" s="24" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
@@ -871,27 +877,27 @@
           <t>TC09</t>
         </is>
       </c>
-      <c r="B12" s="16" t="inlineStr">
+      <c r="B12" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC09</t>
         </is>
       </c>
-      <c r="C12" s="16" t="inlineStr">
+      <c r="C12" s="24" t="inlineStr">
         <is>
           <t>A one-character password is treated as a wrong password, not a malformed one</t>
         </is>
       </c>
-      <c r="D12" s="16" t="inlineStr">
+      <c r="D12" s="24" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="E12" s="16" t="inlineStr">
+      <c r="E12" s="24" t="inlineStr">
         <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="F12" s="16" t="inlineStr">
+      <c r="F12" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -910,27 +916,27 @@
           <t>TC10</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC10</t>
         </is>
       </c>
-      <c r="C13" s="16" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>A deactivated account cannot log in, even with the correct password</t>
         </is>
       </c>
-      <c r="D13" s="16" t="inlineStr">
+      <c r="D13" s="24" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="E13" s="16" t="inlineStr">
+      <c r="E13" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F13" s="16" t="inlineStr">
+      <c r="F13" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -949,27 +955,27 @@
           <t>TC11</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC11</t>
         </is>
       </c>
-      <c r="C14" s="16" t="inlineStr">
+      <c r="C14" s="24" t="inlineStr">
         <is>
           <t>An email typed with different capitalisation</t>
         </is>
       </c>
-      <c r="D14" s="16" t="inlineStr">
+      <c r="D14" s="24" t="inlineStr">
         <is>
           <t>AC1, AC2</t>
         </is>
       </c>
-      <c r="E14" s="16" t="inlineStr">
+      <c r="E14" s="24" t="inlineStr">
         <is>
           <t>Boundary</t>
         </is>
       </c>
-      <c r="F14" s="16" t="inlineStr">
+      <c r="F14" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -988,27 +994,27 @@
           <t>TC12</t>
         </is>
       </c>
-      <c r="B15" s="16" t="inlineStr">
+      <c r="B15" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC12</t>
         </is>
       </c>
-      <c r="C15" s="16" t="inlineStr">
+      <c r="C15" s="24" t="inlineStr">
         <is>
           <t>The signed-in user's role is named on the dashboard</t>
         </is>
       </c>
-      <c r="D15" s="16" t="inlineStr">
+      <c r="D15" s="24" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="E15" s="16" t="inlineStr">
+      <c r="E15" s="24" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F15" s="16" t="inlineStr">
+      <c r="F15" s="24" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
@@ -1027,38 +1033,42 @@
           <t>TC13</t>
         </is>
       </c>
-      <c r="B16" s="16" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC13</t>
         </is>
       </c>
-      <c r="C16" s="16" t="inlineStr">
+      <c r="C16" s="24" t="inlineStr">
         <is>
           <t>The navigation offered matches the role that is signed in</t>
         </is>
       </c>
-      <c r="D16" s="16" t="inlineStr">
+      <c r="D16" s="24" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="E16" s="16" t="inlineStr">
+      <c r="E16" s="24" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F16" s="16" t="inlineStr">
+      <c r="F16" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="H16" s="24" t="n"/>
-      <c r="I16" s="24" t="n"/>
+      <c r="I16" s="24" t="inlineStr">
+        <is>
+          <t>Week 7 #5</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
@@ -1066,27 +1076,27 @@
           <t>TC14</t>
         </is>
       </c>
-      <c r="B17" s="16" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC14</t>
         </is>
       </c>
-      <c r="C17" s="16" t="inlineStr">
+      <c r="C17" s="24" t="inlineStr">
         <is>
           <t>Logging out ends the session</t>
         </is>
       </c>
-      <c r="D17" s="16" t="inlineStr">
+      <c r="D17" s="24" t="inlineStr">
         <is>
           <t>AC3, AC4</t>
         </is>
       </c>
-      <c r="E17" s="16" t="inlineStr">
+      <c r="E17" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F17" s="16" t="inlineStr">
+      <c r="F17" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -1105,27 +1115,27 @@
           <t>TC15</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC15</t>
         </is>
       </c>
-      <c r="C18" s="16" t="inlineStr">
+      <c r="C18" s="24" t="inlineStr">
         <is>
           <t>A signed-out visitor cannot reach a signed-in page</t>
         </is>
       </c>
-      <c r="D18" s="16" t="inlineStr">
+      <c r="D18" s="24" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="E18" s="16" t="inlineStr">
+      <c r="E18" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F18" s="16" t="inlineStr">
+      <c r="F18" s="24" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
@@ -1144,27 +1154,27 @@
           <t>TC16</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC16</t>
         </is>
       </c>
-      <c r="C19" s="16" t="inlineStr">
+      <c r="C19" s="24" t="inlineStr">
         <is>
           <t>A Coordinator cannot raise an event request</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
+      <c r="D19" s="24" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="E19" s="16" t="inlineStr">
+      <c r="E19" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F19" s="16" t="inlineStr">
+      <c r="F19" s="24" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
@@ -1183,38 +1193,42 @@
           <t>TC17</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC17</t>
         </is>
       </c>
-      <c r="C20" s="16" t="inlineStr">
+      <c r="C20" s="24" t="inlineStr">
         <is>
           <t>A stranger cannot give themselves a staff role when registering</t>
         </is>
       </c>
-      <c r="D20" s="16" t="inlineStr">
+      <c r="D20" s="24" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="E20" s="16" t="inlineStr">
+      <c r="E20" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F20" s="16" t="inlineStr">
+      <c r="F20" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
       <c r="G20" s="24" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Updated</t>
         </is>
       </c>
       <c r="H20" s="24" t="n"/>
-      <c r="I20" s="24" t="n"/>
+      <c r="I20" s="24" t="inlineStr">
+        <is>
+          <t>Week 7 #5</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="20">
       <c r="A21" s="9" t="inlineStr">
@@ -1222,27 +1236,27 @@
           <t>TC18</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC18</t>
         </is>
       </c>
-      <c r="C21" s="16" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>An Organiser sees only their own client's events</t>
         </is>
       </c>
-      <c r="D21" s="16" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="E21" s="16" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F21" s="16" t="inlineStr">
+      <c r="F21" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -1261,27 +1275,27 @@
           <t>TC19</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC19</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>A tampered session token is not accepted</t>
         </is>
       </c>
-      <c r="D22" s="16" t="inlineStr">
+      <c r="D22" s="24" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="E22" s="16" t="inlineStr">
+      <c r="E22" s="24" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F22" s="16" t="inlineStr">
+      <c r="F22" s="24" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
@@ -1297,19 +1311,19 @@
     <row r="23" ht="15.75" customHeight="1" s="20"/>
     <row r="24" ht="15.75" customHeight="1" s="20"/>
     <row r="25" ht="15.75" customHeight="1" s="20">
-      <c r="A25" s="1" t="inlineStr">
+      <c r="A25" s="23" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B25" s="1" t="inlineStr">
+      <c r="B25" s="23" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
         </is>
       </c>
       <c r="C25" s="21" t="n"/>
       <c r="D25" s="22" t="n"/>
-      <c r="E25" s="1" t="inlineStr">
+      <c r="E25" s="23" t="inlineStr">
         <is>
           <t>Covered by</t>
         </is>
@@ -1317,19 +1331,19 @@
       <c r="F25" s="22" t="n"/>
     </row>
     <row r="26" ht="71.25" customHeight="1" s="20">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="24" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="B26" s="16" t="inlineStr">
+      <c r="B26" s="24" t="inlineStr">
         <is>
           <t>Given I have valid credentials, when I log in, then I am authenticated successfully.</t>
         </is>
       </c>
       <c r="C26" s="21" t="n"/>
       <c r="D26" s="22" t="n"/>
-      <c r="E26" s="16" t="inlineStr">
+      <c r="E26" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC01
 SPM-21-TC02
@@ -1341,19 +1355,19 @@
       <c r="F26" s="22" t="n"/>
     </row>
     <row r="27" ht="98.25" customHeight="1" s="20">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="24" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B27" s="16" t="inlineStr">
+      <c r="B27" s="24" t="inlineStr">
         <is>
           <t>Given I enter invalid credentials, when I attempt to log in, then access is denied and an appropriate error message is displayed.</t>
         </is>
       </c>
       <c r="C27" s="21" t="n"/>
       <c r="D27" s="22" t="n"/>
-      <c r="E27" s="16" t="inlineStr">
+      <c r="E27" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC05
 SPM-21-TC06
@@ -1367,19 +1381,19 @@
       <c r="F27" s="22" t="n"/>
     </row>
     <row r="28" ht="57.75" customHeight="1" s="20">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="24" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="B28" s="16" t="inlineStr">
+      <c r="B28" s="24" t="inlineStr">
         <is>
           <t>Given I am logged in, when I access the system, then my role is identified.</t>
         </is>
       </c>
       <c r="C28" s="21" t="n"/>
       <c r="D28" s="22" t="n"/>
-      <c r="E28" s="16" t="inlineStr">
+      <c r="E28" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC04
 SPM-21-TC12
@@ -1390,19 +1404,19 @@
       <c r="F28" s="22" t="n"/>
     </row>
     <row r="29" ht="84.75" customHeight="1" s="20">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="24" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="B29" s="16" t="inlineStr">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>Given I am logged in, when I access a function that my role is not authorised for, then access is denied.</t>
         </is>
       </c>
       <c r="C29" s="21" t="n"/>
       <c r="D29" s="22" t="n"/>
-      <c r="E29" s="16" t="inlineStr">
+      <c r="E29" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC14
 SPM-21-TC15
@@ -1416,12 +1430,12 @@
     </row>
     <row r="30" ht="15.75" customHeight="1" s="20"/>
     <row r="31" ht="179.25" customHeight="1" s="20">
-      <c r="A31" s="1" t="inlineStr">
+      <c r="A31" s="23" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B31" s="16" t="inlineStr">
+      <c r="B31" s="24" t="inlineStr">
         <is>
           <t>src/app/api/auth/login/route.ts
 src/app/api/auth/me/route.ts
@@ -2481,7 +2495,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC09</t>
         </is>
@@ -2493,7 +2507,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>No one is signed in. On the "Log in" page.</t>
         </is>
@@ -2505,7 +2519,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "daniel.tan@connectsphere.com" into Email
 2. Enter "x" into Password
@@ -2519,7 +2533,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: daniel.tan@connectsphere.com; Password: x</t>
         </is>
@@ -2531,7 +2545,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The error message is "Invalid email or password" — the shortest allowed password is one character, so the attempt is checked as a credential rather than rejected as an empty field.
 The browser stays on the "Log in" page.</t>
@@ -2544,7 +2558,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -2576,7 +2590,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login with "Invalid email or password" - the same credential refusal as TC05, not the field-level error of TC07/TC08.</t>
         </is>
@@ -2600,7 +2614,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Confirms the boundary: loginSchema allows a one-character password, so a single character is checked as a credential rather than rejected as empty.</t>
         </is>
@@ -2612,7 +2626,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -2644,7 +2658,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login with "Invalid email or password" - the same credential refusal as TC05, not the field-level error of TC07/TC08.</t>
         </is>
@@ -2668,7 +2682,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -2680,7 +2694,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle</t>
         </is>
@@ -3707,7 +3721,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC10</t>
         </is>
@@ -3719,7 +3733,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Marcus Wong (marcus.wong@connectsphere.com) has been deactivated: open Prisma Studio (npx prisma studio), find the row in Users and set Is Active to false. No one is signed in. On the "Log in" page.</t>
         </is>
@@ -3731,7 +3745,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "marcus.wong@connectsphere.com" into Email
 2. Enter "password123" into Password
@@ -3746,7 +3760,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: marcus.wong@connectsphere.com; Password: password123; Is Active: false</t>
         </is>
@@ -3758,7 +3772,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The error message "This account has been deactivated. Contact your ConnectSphere administrator." is shown.
 The browser stays on the "Log in" page and no dashboard is reached.</t>
@@ -3771,7 +3785,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -3803,7 +3817,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>With Marcus Wong set to Is Active = false, logging in with the correct password stayed on /login and showed "This account has been deactivated. Contact your ConnectSphere administrator." No session was created and no sidebar appeared.</t>
         </is>
@@ -3827,7 +3841,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Account reactivated after the run and re-verified: marcus.wong logs in normally again. Note this message does confirm the account exists - a deliberate trade documented in src/app/api/auth/login/route.ts.</t>
         </is>
@@ -3839,7 +3853,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -3871,7 +3885,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>showed "This account has been deactivated. Contact your ConnectSphere administrator." No session was created and no sidebar appeared.</t>
         </is>
@@ -3895,7 +3909,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -3907,7 +3921,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -4934,7 +4948,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC11</t>
         </is>
@@ -4946,7 +4960,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Demo data is seeded. No one is signed in. On the "Log in" page.</t>
         </is>
@@ -4958,7 +4972,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "Daniel.Tan@connectsphere.com" into Email
 2. Enter "password123" into Password
@@ -4972,7 +4986,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: Daniel.Tan@connectsphere.com (same address as TC01, different capitalisation); Password: password123</t>
         </is>
@@ -4984,7 +4998,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The user is signed in and the Dashboard opens, headed "Welcome, Daniel Tan" — an email address is not case sensitive, so this is the same account as TC01.</t>
         </is>
@@ -4996,7 +5010,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -5028,7 +5042,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Signed in successfully. The browser moved to /dashboard headed "Welcome, Daniel Tan" / "Event Coordinator" - the same account TC01 reaches with the all-lowercase address.</t>
         </is>
@@ -5052,7 +5066,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Re-run after the fix. First run on 2026-09-20 FAILED with "Invalid email or password". loginSchema and registerSchema now trim and lower-case the address before it is checked or stored. See Open Questions #2.</t>
         </is>
@@ -5064,7 +5078,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -5095,7 +5109,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Signed in successfully. The browser moved to /dashboard headed "Welcome, Daniel Tan" / "Event Coordinator" - the same account TC01 reaches with the all-lowercase address.</t>
         </is>
@@ -5119,7 +5133,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -5131,7 +5145,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -6159,7 +6173,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC12</t>
         </is>
@@ -6171,7 +6185,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Demo data is seeded. No one is signed in.</t>
         </is>
@@ -6183,7 +6197,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Log in as daniel.tan@connectsphere.com with password123
 2. Read the subtitle under the welcome heading
@@ -6198,7 +6212,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Accounts: daniel.tan@connectsphere.com (Coordinator), marcus.wong@connectsphere.com (Venue Staff); Password: password123</t>
         </is>
@@ -6210,7 +6224,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Daniel Tan's dashboard is headed "Welcome, Daniel Tan", subtitled "Event Coordinator" and the section heading reads "Awaiting your review".
 Marcus Wong's dashboard is headed "Welcome, Marcus Wong", subtitled "Venue Staff" and the section heading reads "Upcoming events".</t>
@@ -6223,7 +6237,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -6255,7 +6269,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Daniel Tan: headed "Welcome, Daniel Tan", subtitled "Event Coordinator", section heading "Awaiting your review". Marcus Wong: headed "Welcome, Marcus Wong", subtitled "Venue Staff", section heading "Upcoming events".</t>
         </is>
@@ -6279,7 +6293,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>The role is identified in two places - the page subtitle and the top bar - and the dashboard content changes with it.</t>
         </is>
@@ -6291,7 +6305,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -6323,7 +6337,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Daniel Tan: headed "Welcome, Daniel Tan", subtitled "Event Coordinator", section heading "Awaiting your review". Marcus Wong: headed "Welcome, Marcus Wong", subtitled "Venue Staff", section heading "Upcoming events".</t>
         </is>
@@ -6347,7 +6361,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -6359,7 +6373,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -7364,7 +7378,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="24.75" customWidth="1" style="20" min="1" max="1"/>
@@ -7372,45 +7386,52 @@
     <col width="12.63" customWidth="1" style="20" min="3" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="20">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="90" customHeight="1" s="20">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>v2 (2026-10-20): The Event Operations Manager is now shown as the 'Event Coordinator Lead' (SPM-84 AC1, forum #129, Week 7 Change #5) - the same role, accounts, permissions and pages. Read 'Operations Manager', 'Event Operations Manager' or 'Ops Manager' in this case as 'Event Coordinator Lead'; on screen the role is shown under its new name, and refusals say 'Assigning coordinators is the Event Coordinator Lead's role.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="17.25" customHeight="1" s="20">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="17.25" customHeight="1" s="20">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="16" t="inlineStr">
-        <is>
-          <t>SPM-21-TC13</t>
-        </is>
-      </c>
+      <c r="B2" s="5" t="n"/>
     </row>
     <row r="3" ht="17.25" customHeight="1" s="20">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>Demo data is seeded. No one is signed in.</t>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>SPM-21-TC13</t>
         </is>
       </c>
     </row>
     <row r="4" ht="71.25" customHeight="1" s="20">
       <c r="A4" s="7" t="inlineStr">
         <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Demo data is seeded. No one is signed in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="44.25" customHeight="1" s="20">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>1. Log in as rachel.ng@meridianfina.com with password123
 2. Write down every item in the sidebar
@@ -7419,25 +7440,25 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="44.25" customHeight="1" s="20">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Accounts: rachel.ng@meridianfina.com (Organiser), grace.lim@connectsphere.com (Operations Manager); Password: password123</t>
-        </is>
-      </c>
-    </row>
     <row r="6" ht="84.75" customHeight="1" s="20">
       <c r="A6" s="7" t="inlineStr">
         <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Accounts: rachel.ng@meridianfina.com (Organiser), grace.lim@connectsphere.com (Operations Manager); Password: password123</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17.25" customHeight="1" s="20">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Rachel Ng's sidebar reads Dashboard, My Events, Notifications.
 Grace Lim's sidebar reads Dashboard, Assignments, All Events, Notifications.
@@ -7445,165 +7466,164 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="17.25" customHeight="1" s="20">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>TAN JORDAN</t>
-        </is>
-      </c>
-    </row>
     <row r="8" ht="15.75" customHeight="1" s="20">
       <c r="A8" s="7" t="inlineStr">
         <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>TAN JORDAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1" s="20">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B9" s="10" t="n">
         <v>46285</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" s="20"/>
-    <row r="10" ht="15.75" customHeight="1" s="20">
-      <c r="A10" s="11" t="inlineStr">
+    <row r="10" ht="15.75" customHeight="1" s="20"/>
+    <row r="11" ht="57.75" customHeight="1" s="20">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="13" t="n"/>
-    </row>
-    <row r="11" ht="57.75" customHeight="1" s="20">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>Rachel Ng (Organiser): Dashboard, My Events, Notifications. Grace Lim (Operations Manager): Dashboard, Assignments, All Events, Notifications. Same chrome, same layout; header read "Welcome, Grace Lim" / "Operations Manager".</t>
-        </is>
-      </c>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="13" t="n"/>
     </row>
     <row r="12" ht="17.25" customHeight="1" s="20">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>Rachel Ng (Organiser): Dashboard, My Events, Notifications. Grace Lim (Operations Manager): Dashboard, Assignments, All Events, Notifications. Same chrome, same layout; header read "Welcome, Grace Lim" / "Operations Manager".</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44.25" customHeight="1" s="20">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>Navigation comes from NAV_BY_ROLE in src/lib/roles.ts. Note several of these items point at screens that are not built yet - see Open Questions #4.</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1" s="20">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t>TAN JORDAN</t>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Navigation comes from NAV_BY_ROLE in src/lib/roles.ts. Note several of these items point at screens that are not built yet - see Open Questions #4.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="20">
       <c r="A15" s="14" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t>TAN JORDAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1" s="20">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B16" s="10" t="n">
         <v>46285</v>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1" s="20"/>
     <row r="17" ht="15.75" customHeight="1" s="20"/>
-    <row r="18" ht="15.75" customHeight="1" s="20">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="18" ht="15.75" customHeight="1" s="20"/>
+    <row r="19" ht="15.75" customHeight="1" s="20">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n"/>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="20">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>Rachel Ng (Event Organiser): Dashboard, My Events, Notifications. Grace Lim (Operations Manager): Dashboard, Assignments, All Events, Notifications. Same chrome, same layout; header read "Welcome, Grace Lim" / "Operations Manager".</t>
-        </is>
-      </c>
+      <c r="B19" s="12" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>Rachel Ng (Event Organiser): Dashboard, My Events, Notifications. Grace Lim (Operations Manager): Dashboard, Assignments, All Events, Notifications. Same chrome, same layout; header read "Welcome, Grace Lim" / "Operations Manager".</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="20">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="20">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>Janelle Ip</t>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="20">
       <c r="A23" s="14" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Janelle Ip</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="20">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B23" s="10" t="n">
+      <c r="B24" s="10" t="n">
         <v>46285</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="20"/>
     <row r="25" ht="15.75" customHeight="1" s="20"/>
     <row r="26" ht="15.75" customHeight="1" s="20"/>
     <row r="27" ht="15.75" customHeight="1" s="20"/>
@@ -8581,6 +8601,9 @@
     <row r="999" ht="15.75" customHeight="1" s="20"/>
     <row r="1000" ht="15.75" customHeight="1" s="20"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
@@ -8614,7 +8637,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC14</t>
         </is>
@@ -8626,7 +8649,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Signed in as Daniel Tan (daniel.tan@connectsphere.com / password123), on the Dashboard.</t>
         </is>
@@ -8638,7 +8661,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Click the account control in the top bar
 2. Click "Log out"
@@ -8652,7 +8675,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Account: daniel.tan@connectsphere.com</t>
         </is>
@@ -8664,7 +8687,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Logging out returns the browser to the "Log in" page and the sidebar disappears.
 Opening the Dashboard again lands back on "Log in" instead of showing Daniel Tan's dashboard.</t>
@@ -8677,7 +8700,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -8709,7 +8732,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Clicking Log out returned the browser to /login/dashboard and the sidebar disappeared. Asking for the Dashboard again landed straight back on the login page.</t>
         </is>
@@ -8733,7 +8756,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>clearToken() notifies every mounted useCurrentUser(), so the chrome drops the session immediately rather than on the next reload.</t>
         </is>
@@ -8745,7 +8768,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -8777,7 +8800,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Clicking Log out returned the browser to /login/dashboard and the sidebar disappeared. Asking for the Dashboard again landed straight back on the login page.</t>
         </is>
@@ -8801,7 +8824,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -8813,7 +8836,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -9840,7 +9863,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC15</t>
         </is>
@@ -9852,7 +9875,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>No one is signed in.</t>
         </is>
@@ -9864,7 +9887,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Open the Dashboard directly in the browser
 2. Observe where the browser lands</t>
@@ -9877,7 +9900,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Page requested: Dashboard, with no session</t>
         </is>
@@ -9889,7 +9912,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The browser is sent to the "Log in" page with the notice "Your session expired. Log in to continue where you left off."
 No dashboard content, event list or role name is shown at any point.</t>
@@ -9902,7 +9925,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -9934,7 +9957,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Requesting the Dashboard with no session landed on /login/dashboard showing "Your session expired. Log in to continue where you left off." No role name and no event title appeared anywhere on the page.</t>
         </is>
@@ -9958,7 +9981,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Checked the whole page body for leaked role names and event headings - none present at any point.</t>
         </is>
@@ -9970,7 +9993,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -10001,7 +10024,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Requesting the Dashboard with no session landed on /login/dashboard showing "Your session expired. Log in to continue where you left off." No role name and no event title appeared anywhere on the page.</t>
         </is>
@@ -10025,7 +10048,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -10037,7 +10060,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -11065,7 +11088,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC16</t>
         </is>
@@ -11077,7 +11100,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Signed in as Daniel Tan (daniel.tan@connectsphere.com / password123), a Coordinator. The sidebar offers no "New request" action.</t>
         </is>
@@ -11089,7 +11112,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Open the "New event request" page directly in the browser
 2. Enter "Coordinator authorisation check" into Event name
@@ -11107,7 +11130,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Account: daniel.tan@connectsphere.com (Coordinator); Event name: Coordinator authorisation check; Expected attendance: 50</t>
         </is>
@@ -11119,7 +11142,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The error message "Only an Event Organiser can raise an event request" is shown above the form.
 The browser stays on the form and no draft is created — opening All Events afterwards shows no event named "Coordinator authorisation check".</t>
@@ -11132,7 +11155,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -11164,7 +11187,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>The form submitted and the browser stayed on /events/new with the alert "Only an Event Organiser can raise an event request". Opening All Events afterwards showed no event named "Coordinator authorisation check".</t>
         </is>
@@ -11188,7 +11211,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>The page has no client-side role gate, so the refusal comes from the server and is surfaced on the form. Nothing was written to the database.</t>
         </is>
@@ -11200,7 +11223,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -11232,7 +11255,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>The form submitted and the browser stayed on /events/new with the alert "Only an Event Organiser can raise an event request". Opening All Events afterwards showed no event named "Coordinator authorisation check".</t>
         </is>
@@ -11256,7 +11279,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>upon clicking submit request, Only an Event Organiser can raise an event request error message is shown at the top but the cursor doesnt move to the top</t>
         </is>
@@ -11268,7 +11291,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -12273,7 +12296,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.63" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="24.75" customWidth="1" style="20" min="1" max="1"/>
@@ -12281,235 +12304,241 @@
     <col width="12.63" customWidth="1" style="20" min="3" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15.75" customHeight="1" s="20">
-      <c r="A1" s="2" t="inlineStr">
+    <row r="1" ht="90" customHeight="1" s="20">
+      <c r="A1" s="25" t="inlineStr">
+        <is>
+          <t>v2 (2026-10-20): The Event Operations Manager is now shown as the 'Event Coordinator Lead' (SPM-84 AC1, forum #129, Week 7 Change #5) - the same role, accounts, permissions and pages. Read 'Operations Manager', 'Event Operations Manager' or 'Ops Manager' in this case as 'Event Coordinator Lead'; on screen the role is shown under its new name, and refusals say 'Assigning coordinators is the Event Coordinator Lead's role.'</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="17.25" customHeight="1" s="20">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="5" t="n"/>
-    </row>
-    <row r="2" ht="17.25" customHeight="1" s="20">
-      <c r="A2" s="7" t="inlineStr">
-        <is>
-          <t>Test Case ID</t>
-        </is>
-      </c>
-      <c r="B2" s="16" t="inlineStr">
-        <is>
-          <t>SPM-21-TC17</t>
-        </is>
-      </c>
+      <c r="B2" s="5" t="n"/>
     </row>
     <row r="3" ht="17.25" customHeight="1" s="20">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Pre-conditions</t>
-        </is>
-      </c>
-      <c r="B3" s="16" t="inlineStr">
-        <is>
-          <t>No one is signed in. On the "Register" page.</t>
+          <t>Test Case ID</t>
+        </is>
+      </c>
+      <c r="B3" s="24" t="inlineStr">
+        <is>
+          <t>SPM-21-TC17</t>
         </is>
       </c>
     </row>
     <row r="4" ht="30.75" customHeight="1" s="20">
       <c r="A4" s="7" t="inlineStr">
         <is>
+          <t>Pre-conditions</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>No one is signed in. On the "Register" page.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="17.25" customHeight="1" s="20">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>1. Open the Role dropdown
 2. Read every option offered</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="17.25" customHeight="1" s="20">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Test Data</t>
-        </is>
-      </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Page: Register</t>
-        </is>
-      </c>
-    </row>
     <row r="6" ht="71.25" customHeight="1" s="20">
       <c r="A6" s="7" t="inlineStr">
         <is>
+          <t>Test Data</t>
+        </is>
+      </c>
+      <c r="B6" s="24" t="inlineStr">
+        <is>
+          <t>Page: Register</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="17.25" customHeight="1" s="20">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>The dropdown offers exactly two options: "Event Organiser" and "Attendee".
 Event Coordinator, Operations Manager, Venue Staff and Technical Support are not offered, so a staff account cannot be created by self-registration.</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="17.25" customHeight="1" s="20">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Created By</t>
-        </is>
-      </c>
-      <c r="B7" s="16" t="inlineStr">
-        <is>
-          <t>TAN JORDAN</t>
-        </is>
-      </c>
-    </row>
     <row r="8" ht="15.75" customHeight="1" s="20">
       <c r="A8" s="7" t="inlineStr">
         <is>
+          <t>Created By</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>TAN JORDAN</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1" s="20">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B9" s="10" t="n">
         <v>46285</v>
       </c>
     </row>
-    <row r="9" ht="15.75" customHeight="1" s="20"/>
-    <row r="10" ht="15.75" customHeight="1" s="20">
-      <c r="A10" s="11" t="inlineStr">
+    <row r="10" ht="15.75" customHeight="1" s="20"/>
+    <row r="11" ht="44.25" customHeight="1" s="20">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n"/>
-      <c r="C10" s="13" t="n"/>
-    </row>
-    <row r="11" ht="44.25" customHeight="1" s="20">
-      <c r="A11" s="14" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B11" s="16" t="inlineStr">
-        <is>
-          <t>The Role dropdown offered exactly two options: "Event Organiser" and "Attendee". No Coordinator, Operations Manager, Venue Staff or Technical Support option was present.</t>
-        </is>
-      </c>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="13" t="n"/>
     </row>
     <row r="12" ht="17.25" customHeight="1" s="20">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B12" s="18" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B12" s="24" t="inlineStr">
+        <is>
+          <t>The Role dropdown offered exactly two options: "Event Organiser" and "Attendee". No Coordinator, Operations Manager, Venue Staff or Technical Support option was present.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44.25" customHeight="1" s="20">
       <c r="A13" s="14" t="inlineStr">
         <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B13" s="16" t="inlineStr">
-        <is>
-          <t>Driven by SELF_REGISTERABLE_ROLES in src/lib/roles.ts, which the register route also enforces server-side - the list is not merely hidden in the UI.</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="14" ht="17.25" customHeight="1" s="20">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B14" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">TAN JORDAN </t>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t>Driven by SELF_REGISTERABLE_ROLES in src/lib/roles.ts, which the register route also enforces server-side - the list is not merely hidden in the UI.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15.75" customHeight="1" s="20">
       <c r="A15" s="14" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B15" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TAN JORDAN </t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1" s="20">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B16" s="10" t="n">
         <v>46285</v>
       </c>
     </row>
-    <row r="16" ht="15.75" customHeight="1" s="20"/>
     <row r="17" ht="15.75" customHeight="1" s="20"/>
-    <row r="18" ht="15.75" customHeight="1" s="20">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="18" ht="15.75" customHeight="1" s="20"/>
+    <row r="19" ht="15.75" customHeight="1" s="20">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B18" s="12" t="n"/>
-    </row>
-    <row r="19" ht="15.75" customHeight="1" s="20">
-      <c r="A19" s="14" t="inlineStr">
-        <is>
-          <t>Actual Result</t>
-        </is>
-      </c>
-      <c r="B19" s="16" t="inlineStr">
-        <is>
-          <t>The Role dropdown offered exactly two options: "Event Organiser" and "Attendee". No Coordinator, Operations Manager, Venue Staff or Technical Support option was present.</t>
-        </is>
-      </c>
+      <c r="B19" s="12" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>Pass/Fail/Not Executed/Blocked</t>
-        </is>
-      </c>
-      <c r="B20" s="18" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="B20" s="24" t="inlineStr">
+        <is>
+          <t>The Role dropdown offered exactly two options: "Event Organiser" and "Attendee". No Coordinator, Operations Manager, Venue Staff or Technical Support option was present.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="20">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>Remarks</t>
-        </is>
-      </c>
-      <c r="B21" s="16" t="inlineStr">
-        <is>
-          <t>NA</t>
+          <t>Pass/Fail/Not Executed/Blocked</t>
+        </is>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="20">
       <c r="A22" s="14" t="inlineStr">
         <is>
-          <t>Executed by</t>
-        </is>
-      </c>
-      <c r="B22" s="16" t="inlineStr">
-        <is>
-          <t>Janelle Ip</t>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="20">
       <c r="A23" s="14" t="inlineStr">
         <is>
+          <t>Executed by</t>
+        </is>
+      </c>
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>Janelle Ip</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1" s="20">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B23" s="10" t="n">
+      <c r="B24" s="10" t="n">
         <v>46285</v>
       </c>
     </row>
-    <row r="24" ht="15.75" customHeight="1" s="20"/>
     <row r="25" ht="15.75" customHeight="1" s="20"/>
     <row r="26" ht="15.75" customHeight="1" s="20"/>
     <row r="27" ht="15.75" customHeight="1" s="20"/>
@@ -13487,6 +13516,9 @@
     <row r="999" ht="15.75" customHeight="1" s="20"/>
     <row r="1000" ht="15.75" customHeight="1" s="20"/>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
 </worksheet>
@@ -13520,7 +13552,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC18</t>
         </is>
@@ -13532,7 +13564,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Signed in as Rachel Ng (rachel.ng@meridianfina.com / password123), an Organiser at Meridian Financial Group. Budi Santoso (budi.santoso@nusantaratec.com) is an Organiser at Nusantara Tech Labs and has events of his own.</t>
         </is>
@@ -13544,7 +13576,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Open My Events
 2. Read the title and client of every event listed
@@ -13559,7 +13591,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Accounts: rachel.ng@meridianfina.com (Meridian Financial Group), budi.santoso@nusantaratec.com (Nusantara Tech Labs); Password: password123</t>
         </is>
@@ -13571,7 +13603,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>Rachel Ng's list contains only Meridian Financial Group events.
 Budi Santoso's list contains only Nusantara Tech Labs events.
@@ -13585,7 +13617,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -13617,7 +13649,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Rachel Ng's My Events listed four events, all Meridian Financial Group (Q1 Investor Update draft, Graduate Recruitment Evening, Compliance Training, Wealth Management Forum). Budi Santoso's listed three, all Nusantara Tech Labs (Product Launch, Overnight Hackathon, Developer Summit). No row appeared in both lists.</t>
         </is>
@@ -13641,7 +13673,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Compared the two lists row by row; the intersection was empty. This is a relationship refusal rather than a role one - see Open Questions #5.</t>
         </is>
@@ -13653,7 +13685,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -13685,7 +13717,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Rachel Ng's My Events listed four events, all Meridian Financial Group (Q1 Investor Update draft, Graduate Recruitment Evening, Compliance Training, Wealth Management Forum). Budi Santoso's listed three, all Nusantara Tech Labs (Product Launch, Overnight Hackathon, Developer Summit). No row appeared in both lists.</t>
         </is>
@@ -13709,7 +13741,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -13721,7 +13753,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -14748,7 +14780,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC01</t>
         </is>
@@ -14760,7 +14792,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Demo data is seeded. No one is signed in. On the "Log in" page.</t>
         </is>
@@ -14772,7 +14804,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "daniel.tan@connectsphere.com" into Email
 2. Enter "password123" into Password
@@ -14786,7 +14818,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: daniel.tan@connectsphere.com; Password: password123</t>
         </is>
@@ -14798,7 +14830,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The button shows "Logging in…" while the request is in flight.
 The browser moves to the Dashboard, headed "Welcome, Daniel Tan" with "Event Coordinator" beneath it, and the top bar shows the same role under the name.
@@ -14812,7 +14844,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -14844,7 +14876,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Browser moved to /dashboard. Page headed "Welcome, Daniel Tan" with "Event Coordinator" directly beneath it; the top bar also shows "Daniel Tan" over "Event Coordinator". No error alert. Sidebar: Dashboard, Review Queue, All Events, Venues, Equipment, Notifications.</t>
         </is>
@@ -14868,7 +14900,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Only informational alerts present (the teal "Internal view" note). The "Awaiting your review" cards render as skeletons for about a second before the seeded events appear - a loading state, not an error.</t>
         </is>
@@ -14880,7 +14912,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -14912,7 +14944,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Browser moved to /dashboard. Page headed "Welcome, Daniel Tan" with "Event Coordinator" directly beneath it; the top bar also shows "Daniel Tan" over "Event Coordinator". No error alert. Sidebar: Dashboard, Review Queue, All Events, Venues, Equipment, Notifications.</t>
         </is>
@@ -14936,7 +14968,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>If im previously on events page, logged out and logged back in, i will get redirected to the events page again</t>
         </is>
@@ -14948,7 +14980,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -15975,7 +16007,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC19</t>
         </is>
@@ -15987,7 +16019,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Signed in as Daniel Tan (daniel.tan@connectsphere.com / password123), on the Dashboard.</t>
         </is>
@@ -15999,7 +16031,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Open the browser's developer tools and go to Application, then Local Storage
 2. Change the last five characters of the value stored under "connectsphere_token"
@@ -16013,7 +16045,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Stored key: connectsphere_token, with its last five characters altered</t>
         </is>
@@ -16025,7 +16057,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The browser is sent to the "Log in" page.
 No dashboard content or role name is shown — an altered token is treated as no session at all, not as a valid one.</t>
@@ -16038,7 +16070,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -16070,7 +16102,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>After altering the last five characters of connectsphere_token in Local Storage and reloading, the browser was sent to /login?next=%2Fdashboard. No role name and no dashboard content appeared.</t>
         </is>
@@ -16094,7 +16126,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>The signature no longer verifies, so getActor() returns null and the route answers 401 - an altered token is treated as no session, never as a valid one.</t>
         </is>
@@ -16106,7 +16138,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -16138,7 +16170,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">"The browser is sent to the ""Log in"" page with "Your session expired. Log in to continue where you left off." above the email
 </t>
@@ -16163,7 +16195,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -16175,7 +16207,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -17202,7 +17234,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC02</t>
         </is>
@@ -17214,7 +17246,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>No one is signed in. On the "Log in" page, where no sidebar is shown.</t>
         </is>
@@ -17226,7 +17258,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "rachel.ng@meridianfina.com" into Email
 2. Enter "password123" into Password
@@ -17241,7 +17273,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: rachel.ng@meridianfina.com; Password: password123</t>
         </is>
@@ -17253,7 +17285,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The sidebar appears straight away with Dashboard, My Events and Notifications, and the top bar shows Rachel Ng.
 No browser reload is needed to make the sidebar appear.</t>
@@ -17266,7 +17298,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -17298,7 +17330,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Before logging in the page had no sidebar at all. Immediately after clicking Log in - with no reload - the sidebar rendered "Dashboard, My Events, Notifications" and the top bar showed Rachel Ng. Header read "Welcome, Rachel Ng" / "Event Organiser".</t>
         </is>
@@ -17322,7 +17354,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Confirms the onTokenChange fix in src/lib/session.ts: the already-mounted shell picks up the new session without a page reload.</t>
         </is>
@@ -17334,7 +17366,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -17366,7 +17398,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Before logging in the page had no sidebar at all. Immediately after clicking Log in - with no reload - the sidebar rendered "Dashboard, My Events, Notifications" and the top bar showed Rachel Ng. Header read "Welcome, Rachel Ng" / "Event Organiser".</t>
         </is>
@@ -17390,7 +17422,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -17402,7 +17434,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -18429,7 +18461,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC03</t>
         </is>
@@ -18441,7 +18473,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>No one is signed in.</t>
         </is>
@@ -18453,7 +18485,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Open the My Events page directly in the browser
 2. Observe the page the browser lands on
@@ -18469,7 +18501,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: rachel.ng@meridianfina.com; Password: password123</t>
         </is>
@@ -18481,7 +18513,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The browser lands on the "Log in" page showing the notice "Your session expired. Log in to continue where you left off."
 After logging in, the browser opens My Events, not the Dashboard.</t>
@@ -18494,7 +18526,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -18526,7 +18558,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Requesting My Events while signed out landed on /login?next=%2Fevents showing "Your session expired. Log in to continue where you left off." After logging in, the browser opened /events, headed "My events" - not the Dashboard.</t>
         </is>
@@ -18550,7 +18582,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Return path preserved through the ?next= parameter as specified in UI_DESIGN.md section 7.4.</t>
         </is>
@@ -18562,7 +18594,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -18594,7 +18626,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Requesting My Events while signed out landed on /login?next=%2Fevents showing "Your session expired. Log in to continue where you left off." After logging in, the browser opened /events, headed "My events" - not the Dashboard.</t>
         </is>
@@ -18618,7 +18650,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -18630,7 +18662,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -19657,7 +19689,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC04</t>
         </is>
@@ -19669,7 +19701,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Signed in as Daniel Tan (daniel.tan@connectsphere.com / password123), on the Dashboard.</t>
         </is>
@@ -19681,7 +19713,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Press F5 to reload the page
 2. Wait for the page to finish loading</t>
@@ -19694,7 +19726,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Account: daniel.tan@connectsphere.com</t>
         </is>
@@ -19706,7 +19738,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The Dashboard reloads still signed in as Daniel Tan, still labelled "Event Coordinator".
 The browser is not sent back to the "Log in" page.</t>
@@ -19719,7 +19751,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -19751,7 +19783,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Before reload: "Welcome, Daniel Tan" / "Event Coordinator". After F5 the URL was still /dashboard, the header still read "Welcome, Daniel Tan" / "Event Coordinator", and the Coordinator sidebar was intact. No redirect to the login page.</t>
         </is>
@@ -19775,7 +19807,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Session token survives in localStorage; the role is re-fetched from /api/auth/me rather than trusted from the page.</t>
         </is>
@@ -19787,7 +19819,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -19819,7 +19851,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B19" s="16" t="inlineStr">
+      <c r="B19" s="24" t="inlineStr">
         <is>
           <t>Before reload: "Welcome, Daniel Tan" / "Event Coordinator". After F5 the URL was still /dashboard, the header still read "Welcome, Daniel Tan" / "Event Coordinator", and the Coordinator sidebar was intact. No redirect to the login page.</t>
         </is>
@@ -19843,7 +19875,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -19855,7 +19887,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B22" s="16" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Janelle</t>
         </is>
@@ -20882,7 +20914,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC05</t>
         </is>
@@ -20894,7 +20926,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Demo data is seeded. No one is signed in. On the "Log in" page.</t>
         </is>
@@ -20906,7 +20938,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "daniel.tan@connectsphere.com" into Email
 2. Enter "wrongpass" into Password
@@ -20920,7 +20952,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: daniel.tan@connectsphere.com; Password: wrongpass</t>
         </is>
@@ -20932,7 +20964,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>A red error message "Invalid email or password" is shown above the form.
 The browser stays on the "Log in" page and no sidebar appears.</t>
@@ -20945,7 +20977,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -20977,7 +21009,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login. A red alert reading exactly "Invalid email or password" appeared above the form. No sidebar appeared and no dashboard was reached.</t>
         </is>
@@ -21001,7 +21033,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -21013,7 +21045,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -21044,7 +21076,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login. A red alert reading exactly "Invalid email or password" appeared above the form. No sidebar appeared and no dashboard was reached.</t>
         </is>
@@ -21068,7 +21100,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -21080,7 +21112,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -22108,7 +22140,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC06</t>
         </is>
@@ -22120,7 +22152,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>No account exists for nobody@connectsphere.com. No one is signed in. On the "Log in" page.</t>
         </is>
@@ -22132,7 +22164,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "nobody@connectsphere.com" into Email
 2. Enter "password123" into Password
@@ -22147,7 +22179,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: nobody@connectsphere.com; Password: password123</t>
         </is>
@@ -22159,7 +22191,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The error message is "Invalid email or password" — word for word the same as TC05.
 Nothing on screen reveals whether the account exists.</t>
@@ -22172,7 +22204,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -22204,7 +22236,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login with the alert "Invalid email or password" - character for character the same message TC05 produced for a real account with a wrong password.</t>
         </is>
@@ -22228,7 +22260,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>No account enumeration: the screen gives away nothing about whether nobody@connectsphere.com exists.</t>
         </is>
@@ -22240,7 +22272,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -22271,7 +22303,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login with the alert "Invalid email or password" - character for character the same message TC05 produced for a real account with a wrong password.</t>
         </is>
@@ -22295,7 +22327,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -22307,7 +22339,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>
@@ -23335,7 +23367,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC07</t>
         </is>
@@ -23347,7 +23379,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>No one is signed in. On the "Log in" page.</t>
         </is>
@@ -23359,7 +23391,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "daniel.tan" into Email
 2. Enter "password123" into Password
@@ -23373,7 +23405,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: daniel.tan; Password: password123</t>
         </is>
@@ -23385,7 +23417,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The message "Enter a valid email address" is shown against the Email field, which is outlined in red, so the user can see exactly which field to correct.
 The browser stays on the "Log in" page.</t>
@@ -23398,7 +23430,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -23430,7 +23462,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login. The message "Enter a valid email address" appeared directly under the Email field, with the field outlined in red. No generic banner.</t>
         </is>
@@ -23454,7 +23486,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Re-run after the fix. First run on 2026-09-20 FAILED, showing only "Validation failed" with nothing marking the field. src/app/login/page.tsx now maps the server's fieldErrors through readServerError(). See Open Questions #1.</t>
         </is>
@@ -23466,7 +23498,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -23497,7 +23529,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login. The message "Enter a valid email address" appeared directly under the Email field, with the field outlined in red. No generic banner.</t>
         </is>
@@ -23521,7 +23553,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -24561,7 +24593,7 @@
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="16" t="inlineStr">
+      <c r="B2" s="24" t="inlineStr">
         <is>
           <t>SPM-21-TC08</t>
         </is>
@@ -24573,7 +24605,7 @@
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B3" s="16" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>No one is signed in. On the "Log in" page.</t>
         </is>
@@ -24585,7 +24617,7 @@
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>1. Enter "daniel.tan@connectsphere.com" into Email
 2. Leave Password empty
@@ -24599,7 +24631,7 @@
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
         <is>
           <t>Email: daniel.tan@connectsphere.com; Password: (empty)</t>
         </is>
@@ -24611,7 +24643,7 @@
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>The message "Enter your password" is shown against the Password field, which is outlined in red.
 The browser stays on the "Log in" page.</t>
@@ -24624,7 +24656,7 @@
           <t>Created By</t>
         </is>
       </c>
-      <c r="B7" s="16" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>TAN JORDAN</t>
         </is>
@@ -24656,7 +24688,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B11" s="16" t="inlineStr">
+      <c r="B11" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login. The message "Enter your password" appeared directly under the Password field, with the field outlined in red.</t>
         </is>
@@ -24680,7 +24712,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B13" s="16" t="inlineStr">
+      <c r="B13" s="24" t="inlineStr">
         <is>
           <t>Re-run after the same fix; first run FAILED with a bare "Validation failed". loginSchema now carries a written message instead of Zod's default "String must contain at least 1 character(s)".</t>
         </is>
@@ -24692,7 +24724,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B14" s="16" t="inlineStr">
+      <c r="B14" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">TAN JORDAN </t>
         </is>
@@ -24723,7 +24755,7 @@
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B18" s="16" t="inlineStr">
+      <c r="B18" s="24" t="inlineStr">
         <is>
           <t>Stayed on /login. The message "Enter your password" appeared directly under the Password field, with the field outlined in red.</t>
         </is>
@@ -24747,7 +24779,7 @@
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B20" s="16" t="inlineStr">
+      <c r="B20" s="24" t="inlineStr">
         <is>
           <t>NA</t>
         </is>
@@ -24759,7 +24791,7 @@
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B21" s="16" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>Janelle Ip</t>
         </is>

</xml_diff>